<commit_message>
docs: add NOTE-008 — COV sequence execution order and dependencies
Defines the required regression test execution order for all 19 COV
sequences across Phase 1 (register-only, AXI-Lite) and Phase 2
(UART functional, requires serial driver extension). Documents hard
dependencies between sequences to prevent false failures from
out-of-order execution.

Author: S. Belvin, BelTech Systems LLC
</commit_message>
<xml_diff>
--- a/ip/buffered_axi_lite_uart/buffered_axi_lite_uart_vplan.xlsx
+++ b/ip/buffered_axi_lite_uart/buffered_axi_lite_uart_vplan.xlsx
@@ -152,7 +152,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -235,6 +235,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -17953,7 +17956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -18142,6 +18145,87 @@
       <c r="D9" s="16" t="inlineStr">
         <is>
           <t>UART-BR-004, COV-013</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>NOTE-008</t>
+        </is>
+      </c>
+      <c r="B10" s="35" t="inlineStr">
+        <is>
+          <t>Regression Execution Order</t>
+        </is>
+      </c>
+      <c r="C10" s="35" t="inlineStr">
+        <is>
+          <t>COV sequence execution order in the regression test is defined here and must be followed. Dependencies exist between sequences; executing out of order may produce false failures or miss coverage.
+Phase 1 — Register verification (AXI-Lite reads/writes only):
+  1.  COV-015  RESET_VALUES
+          Must run first. Verifies reset state of all registers before
+          any write modifies them. No prerequisites.
+  2.  COV-014  SCRATCH
+          Run early while register state is clean. No prerequisites.
+  3.  COV-018  READONLY_IGNORE
+          Verifies writes to RO registers are ignored. Must run before
+          any sequence that relies on RO register values being
+          predictable. No prerequisites beyond reset state.
+  4.  COV-016  UART_EN_CONTROL
+          Enables and disables UART_EN, TX_EN, RX_EN, LOOP_EN.
+          Must run before COV-013. Leaves UART_EN=0 at completion.
+  5.  COV-013  BAUD_TUNING_WRITE_WHILE_ENABLED
+          Verifies BAUD_TUNING write is ignored while UART_EN=1.
+          Depends on COV-016. Must leave UART_EN=0 at completion.
+  6.  COV-001  BAUD_TUNING
+          12-value NCO tuning word sweep. Depends on UART_EN=0
+          (writes ignored while enabled per UART-BR-004).
+          Already implemented in seq_RCOV001_baud_tuning.sv.
+  7.  COV-010  AXI_BRESP
+          Verifies AXI write response codes. No state prerequisites
+          beyond UART being in a known state.
+  8.  COV-011  AXI_RRESP
+          Verifies AXI read response codes. Same prerequisites as COV-010.
+  9.  COV-012  AXI_WRITE_ORDER
+          Verifies AW/W channel ordering. Structural AXI-Lite test.
+          No state prerequisites.
+Phase 2 — UART functional (requires UART serial activity on
+uart_tx / uart_rx — driver extension needed before these run):
+  10. COV-017  FRAME_STRUCTURAL
+          First UART framing sequence. Must run before FIFO-level sequences.
+  11. COV-003  CTRL.STOP_BITS
+          Stop bit configuration. Requires UART framing active. Depends on COV-017.
+  12. COV-002  CTRL.PARITY
+          Parity configuration sweep. Requires UART framing active. Depends on COV-017.
+  13. COV-005  FIFO_STATUS.TX_LEVEL
+          TX FIFO occupancy sweep. Requires UART TX active. Depends on COV-017.
+  14. COV-004  FIFO_STATUS.RX_LEVEL
+          RX FIFO occupancy sweep. Requires UART RX active. Depends on COV-017.
+  15. COV-006  TIMEOUT_VAL
+          Receive timeout sweep. Requires RX activity. Depends on COV-004.
+  16. COV-019  INT_THRESH_FRAME
+          Interrupt threshold and frame error coverage.
+          Depends on COV-005, COV-004, COV-006.
+  17. COV-007  INT_STATUS each_bit_independently
+          Each interrupt source fired individually.
+          Depends on COV-019 establishing interrupt infrastructure.
+  18. COV-009  INT_STATUS.TIMEOUT &amp;&amp; INT_STATUS.RX_THRESH
+          Combined timeout and RX threshold interrupt.
+          Depends on COV-006, COV-007.
+  19. COV-008  INT_STATUS.OVERRUN &amp;&amp; INT_STATUS.RX_FULL
+          Overrun and RX full combined. Depends on COV-004, COV-007.
+Smoke test (buffered_axi_lite_uart_smoke_test) runs independently
+of this order and is not part of the regression sequence.
+UART-BR-004 (intentional gap): BAUD_TUNING write-while-enabled
+behavior is partially covered by COV-013. The intentional gap
+noted in the VPR refers to the sub-cycle timing aspect which
+remains deferred.</t>
+        </is>
+      </c>
+      <c r="D10" s="35" t="inlineStr">
+        <is>
+          <t>COV-001, COV-002, COV-003, COV-004, COV-005, COV-006, COV-007, COV-008, COV-009, COV-010, COV-011, COV-012, COV-013, COV-014, COV-015, COV-016, COV-017, COV-018, COV-019</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: resolve vplan path before --collect-results early return
config.py reads [input] vplan from pssgen.toml and maps it to
vplan_file arg. JobSpec gains vplan_file field; orchestrator sets
vplan_path = job.vplan_file or intent_path so the .xlsx path is
resolved before the collect_results block checks it. CLI adds
--vplan PATH flag for explicit override. Fixes the silent skip
of VPR write-back when vplan lives in pssgen.toml rather than
being auto-detected. Also fixes two Windows console UnicodeEncodeError
occurrences (U+2192 arrow replaced with ASCII ->).

250 tests pass. E2e smoke test confirmed: 139 rows updated,
gap_report.json written.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ip/buffered_axi_lite_uart/buffered_axi_lite_uart_vplan.xlsx
+++ b/ip/buffered_axi_lite_uart/buffered_axi_lite_uart_vplan.xlsx
@@ -1133,12 +1133,24 @@
       </c>
       <c r="S4" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T4" s="16" t="inlineStr"/>
-      <c r="U4" s="16" t="inlineStr"/>
-      <c r="V4" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T4" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U4" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V4" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W4" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -1246,12 +1258,24 @@
       </c>
       <c r="S5" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T5" s="16" t="inlineStr"/>
-      <c r="U5" s="16" t="inlineStr"/>
-      <c r="V5" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T5" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U5" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V5" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W5" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -1472,12 +1496,24 @@
       </c>
       <c r="S7" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T7" s="16" t="inlineStr"/>
-      <c r="U7" s="16" t="inlineStr"/>
-      <c r="V7" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T7" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U7" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V7" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W7" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -1585,12 +1621,24 @@
       </c>
       <c r="S8" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T8" s="16" t="inlineStr"/>
-      <c r="U8" s="16" t="inlineStr"/>
-      <c r="V8" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T8" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U8" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V8" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W8" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -1698,12 +1746,24 @@
       </c>
       <c r="S9" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T9" s="16" t="inlineStr"/>
-      <c r="U9" s="16" t="inlineStr"/>
-      <c r="V9" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T9" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U9" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V9" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W9" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -1811,12 +1871,24 @@
       </c>
       <c r="S10" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T10" s="16" t="inlineStr"/>
-      <c r="U10" s="16" t="inlineStr"/>
-      <c r="V10" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T10" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U10" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V10" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W10" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -1924,12 +1996,24 @@
       </c>
       <c r="S11" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T11" s="16" t="inlineStr"/>
-      <c r="U11" s="16" t="inlineStr"/>
-      <c r="V11" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T11" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U11" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V11" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W11" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -2037,12 +2121,24 @@
       </c>
       <c r="S12" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T12" s="16" t="inlineStr"/>
-      <c r="U12" s="16" t="inlineStr"/>
-      <c r="V12" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T12" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U12" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V12" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W12" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -2150,12 +2246,24 @@
       </c>
       <c r="S13" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T13" s="16" t="inlineStr"/>
-      <c r="U13" s="16" t="inlineStr"/>
-      <c r="V13" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T13" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U13" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V13" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W13" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -2263,12 +2371,24 @@
       </c>
       <c r="S14" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T14" s="16" t="inlineStr"/>
-      <c r="U14" s="16" t="inlineStr"/>
-      <c r="V14" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T14" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U14" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V14" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W14" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -2376,12 +2496,24 @@
       </c>
       <c r="S15" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T15" s="16" t="inlineStr"/>
-      <c r="U15" s="16" t="inlineStr"/>
-      <c r="V15" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T15" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U15" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V15" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W15" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -2489,12 +2621,24 @@
       </c>
       <c r="S16" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T16" s="16" t="inlineStr"/>
-      <c r="U16" s="16" t="inlineStr"/>
-      <c r="V16" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T16" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U16" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V16" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W16" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -2602,12 +2746,24 @@
       </c>
       <c r="S17" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T17" s="16" t="inlineStr"/>
-      <c r="U17" s="16" t="inlineStr"/>
-      <c r="V17" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T17" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U17" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V17" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W17" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -2715,12 +2871,24 @@
       </c>
       <c r="S18" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T18" s="16" t="inlineStr"/>
-      <c r="U18" s="16" t="inlineStr"/>
-      <c r="V18" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T18" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U18" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V18" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W18" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -2828,12 +2996,24 @@
       </c>
       <c r="S19" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T19" s="16" t="inlineStr"/>
-      <c r="U19" s="16" t="inlineStr"/>
-      <c r="V19" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T19" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U19" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V19" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W19" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -2941,12 +3121,24 @@
       </c>
       <c r="S20" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T20" s="16" t="inlineStr"/>
-      <c r="U20" s="16" t="inlineStr"/>
-      <c r="V20" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T20" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U20" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V20" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W20" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -3054,12 +3246,24 @@
       </c>
       <c r="S21" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T21" s="16" t="inlineStr"/>
-      <c r="U21" s="16" t="inlineStr"/>
-      <c r="V21" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T21" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U21" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V21" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W21" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -3167,12 +3371,24 @@
       </c>
       <c r="S22" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T22" s="16" t="inlineStr"/>
-      <c r="U22" s="16" t="inlineStr"/>
-      <c r="V22" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T22" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U22" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V22" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W22" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -3280,12 +3496,24 @@
       </c>
       <c r="S23" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T23" s="16" t="inlineStr"/>
-      <c r="U23" s="16" t="inlineStr"/>
-      <c r="V23" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T23" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U23" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V23" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W23" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -3393,12 +3621,24 @@
       </c>
       <c r="S24" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T24" s="16" t="inlineStr"/>
-      <c r="U24" s="16" t="inlineStr"/>
-      <c r="V24" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T24" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U24" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V24" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W24" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -3506,12 +3746,24 @@
       </c>
       <c r="S25" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T25" s="16" t="inlineStr"/>
-      <c r="U25" s="16" t="inlineStr"/>
-      <c r="V25" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T25" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U25" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V25" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W25" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -3619,12 +3871,24 @@
       </c>
       <c r="S26" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T26" s="16" t="inlineStr"/>
-      <c r="U26" s="16" t="inlineStr"/>
-      <c r="V26" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T26" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U26" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V26" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W26" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -3732,12 +3996,24 @@
       </c>
       <c r="S27" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T27" s="16" t="inlineStr"/>
-      <c r="U27" s="16" t="inlineStr"/>
-      <c r="V27" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T27" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U27" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V27" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W27" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -3845,12 +4121,24 @@
       </c>
       <c r="S28" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T28" s="16" t="inlineStr"/>
-      <c r="U28" s="16" t="inlineStr"/>
-      <c r="V28" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T28" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U28" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V28" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W28" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -3958,12 +4246,24 @@
       </c>
       <c r="S29" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T29" s="16" t="inlineStr"/>
-      <c r="U29" s="16" t="inlineStr"/>
-      <c r="V29" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T29" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U29" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V29" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W29" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -4071,12 +4371,24 @@
       </c>
       <c r="S30" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T30" s="16" t="inlineStr"/>
-      <c r="U30" s="16" t="inlineStr"/>
-      <c r="V30" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T30" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U30" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V30" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W30" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -4184,12 +4496,24 @@
       </c>
       <c r="S31" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T31" s="16" t="inlineStr"/>
-      <c r="U31" s="16" t="inlineStr"/>
-      <c r="V31" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T31" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U31" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V31" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W31" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -4297,12 +4621,24 @@
       </c>
       <c r="S32" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T32" s="16" t="inlineStr"/>
-      <c r="U32" s="16" t="inlineStr"/>
-      <c r="V32" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T32" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U32" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V32" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W32" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -4410,12 +4746,24 @@
       </c>
       <c r="S33" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T33" s="16" t="inlineStr"/>
-      <c r="U33" s="16" t="inlineStr"/>
-      <c r="V33" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T33" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U33" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V33" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W33" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -4523,12 +4871,24 @@
       </c>
       <c r="S34" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T34" s="16" t="inlineStr"/>
-      <c r="U34" s="16" t="inlineStr"/>
-      <c r="V34" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T34" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U34" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V34" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W34" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -4636,12 +4996,24 @@
       </c>
       <c r="S35" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T35" s="16" t="inlineStr"/>
-      <c r="U35" s="16" t="inlineStr"/>
-      <c r="V35" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T35" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U35" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V35" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W35" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -4741,12 +5113,24 @@
       </c>
       <c r="S36" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T36" s="16" t="inlineStr"/>
-      <c r="U36" s="16" t="inlineStr"/>
-      <c r="V36" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T36" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U36" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V36" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W36" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -4854,12 +5238,24 @@
       </c>
       <c r="S37" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T37" s="16" t="inlineStr"/>
-      <c r="U37" s="16" t="inlineStr"/>
-      <c r="V37" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T37" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U37" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V37" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W37" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -4967,12 +5363,24 @@
       </c>
       <c r="S38" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T38" s="16" t="inlineStr"/>
-      <c r="U38" s="16" t="inlineStr"/>
-      <c r="V38" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T38" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U38" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V38" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W38" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -5080,12 +5488,24 @@
       </c>
       <c r="S39" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T39" s="16" t="inlineStr"/>
-      <c r="U39" s="16" t="inlineStr"/>
-      <c r="V39" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T39" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U39" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V39" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W39" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -5193,12 +5613,24 @@
       </c>
       <c r="S40" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T40" s="16" t="inlineStr"/>
-      <c r="U40" s="16" t="inlineStr"/>
-      <c r="V40" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T40" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U40" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V40" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W40" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -5306,12 +5738,24 @@
       </c>
       <c r="S41" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T41" s="16" t="inlineStr"/>
-      <c r="U41" s="16" t="inlineStr"/>
-      <c r="V41" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T41" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U41" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V41" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W41" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -5419,12 +5863,24 @@
       </c>
       <c r="S42" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T42" s="16" t="inlineStr"/>
-      <c r="U42" s="16" t="inlineStr"/>
-      <c r="V42" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T42" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U42" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V42" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W42" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -5532,12 +5988,24 @@
       </c>
       <c r="S43" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T43" s="16" t="inlineStr"/>
-      <c r="U43" s="16" t="inlineStr"/>
-      <c r="V43" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T43" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U43" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V43" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W43" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -5645,12 +6113,24 @@
       </c>
       <c r="S44" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T44" s="16" t="inlineStr"/>
-      <c r="U44" s="16" t="inlineStr"/>
-      <c r="V44" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T44" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U44" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V44" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W44" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -5758,12 +6238,24 @@
       </c>
       <c r="S45" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T45" s="16" t="inlineStr"/>
-      <c r="U45" s="16" t="inlineStr"/>
-      <c r="V45" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T45" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U45" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V45" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W45" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -5871,12 +6363,24 @@
       </c>
       <c r="S46" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T46" s="16" t="inlineStr"/>
-      <c r="U46" s="16" t="inlineStr"/>
-      <c r="V46" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T46" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U46" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V46" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W46" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -5984,12 +6488,24 @@
       </c>
       <c r="S47" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T47" s="16" t="inlineStr"/>
-      <c r="U47" s="16" t="inlineStr"/>
-      <c r="V47" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T47" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U47" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V47" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W47" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -6097,12 +6613,24 @@
       </c>
       <c r="S48" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T48" s="16" t="inlineStr"/>
-      <c r="U48" s="16" t="inlineStr"/>
-      <c r="V48" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T48" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U48" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V48" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W48" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -6210,12 +6738,24 @@
       </c>
       <c r="S49" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T49" s="16" t="inlineStr"/>
-      <c r="U49" s="16" t="inlineStr"/>
-      <c r="V49" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T49" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U49" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V49" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W49" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -6323,12 +6863,24 @@
       </c>
       <c r="S50" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T50" s="16" t="inlineStr"/>
-      <c r="U50" s="16" t="inlineStr"/>
-      <c r="V50" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T50" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U50" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V50" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W50" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -6436,12 +6988,24 @@
       </c>
       <c r="S51" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T51" s="16" t="inlineStr"/>
-      <c r="U51" s="16" t="inlineStr"/>
-      <c r="V51" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T51" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U51" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V51" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W51" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -6549,12 +7113,24 @@
       </c>
       <c r="S52" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T52" s="16" t="inlineStr"/>
-      <c r="U52" s="16" t="inlineStr"/>
-      <c r="V52" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T52" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U52" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V52" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W52" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -6662,12 +7238,24 @@
       </c>
       <c r="S53" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T53" s="16" t="inlineStr"/>
-      <c r="U53" s="16" t="inlineStr"/>
-      <c r="V53" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T53" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U53" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V53" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W53" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -6775,12 +7363,24 @@
       </c>
       <c r="S54" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T54" s="16" t="inlineStr"/>
-      <c r="U54" s="16" t="inlineStr"/>
-      <c r="V54" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T54" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U54" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V54" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W54" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -6888,12 +7488,24 @@
       </c>
       <c r="S55" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T55" s="16" t="inlineStr"/>
-      <c r="U55" s="16" t="inlineStr"/>
-      <c r="V55" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T55" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U55" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V55" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W55" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -7001,12 +7613,24 @@
       </c>
       <c r="S56" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T56" s="16" t="inlineStr"/>
-      <c r="U56" s="16" t="inlineStr"/>
-      <c r="V56" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T56" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U56" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V56" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W56" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -7114,12 +7738,24 @@
       </c>
       <c r="S57" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T57" s="16" t="inlineStr"/>
-      <c r="U57" s="16" t="inlineStr"/>
-      <c r="V57" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T57" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U57" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V57" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W57" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -7227,12 +7863,24 @@
       </c>
       <c r="S58" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T58" s="16" t="inlineStr"/>
-      <c r="U58" s="16" t="inlineStr"/>
-      <c r="V58" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T58" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U58" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V58" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W58" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -7340,12 +7988,24 @@
       </c>
       <c r="S59" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T59" s="16" t="inlineStr"/>
-      <c r="U59" s="16" t="inlineStr"/>
-      <c r="V59" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T59" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U59" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V59" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W59" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -7453,12 +8113,24 @@
       </c>
       <c r="S60" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T60" s="16" t="inlineStr"/>
-      <c r="U60" s="16" t="inlineStr"/>
-      <c r="V60" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T60" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U60" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V60" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W60" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -7566,12 +8238,24 @@
       </c>
       <c r="S61" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T61" s="16" t="inlineStr"/>
-      <c r="U61" s="16" t="inlineStr"/>
-      <c r="V61" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T61" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U61" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V61" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W61" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -7679,12 +8363,24 @@
       </c>
       <c r="S62" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T62" s="16" t="inlineStr"/>
-      <c r="U62" s="16" t="inlineStr"/>
-      <c r="V62" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T62" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U62" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V62" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W62" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -7792,12 +8488,24 @@
       </c>
       <c r="S63" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T63" s="16" t="inlineStr"/>
-      <c r="U63" s="16" t="inlineStr"/>
-      <c r="V63" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T63" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U63" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V63" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W63" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -7905,12 +8613,24 @@
       </c>
       <c r="S64" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T64" s="16" t="inlineStr"/>
-      <c r="U64" s="16" t="inlineStr"/>
-      <c r="V64" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T64" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U64" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V64" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W64" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -8018,12 +8738,24 @@
       </c>
       <c r="S65" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T65" s="16" t="inlineStr"/>
-      <c r="U65" s="16" t="inlineStr"/>
-      <c r="V65" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T65" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U65" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V65" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W65" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -8131,12 +8863,24 @@
       </c>
       <c r="S66" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T66" s="16" t="inlineStr"/>
-      <c r="U66" s="16" t="inlineStr"/>
-      <c r="V66" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T66" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U66" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V66" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W66" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -8244,12 +8988,24 @@
       </c>
       <c r="S67" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T67" s="16" t="inlineStr"/>
-      <c r="U67" s="16" t="inlineStr"/>
-      <c r="V67" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T67" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U67" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V67" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W67" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -8357,12 +9113,24 @@
       </c>
       <c r="S68" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T68" s="16" t="inlineStr"/>
-      <c r="U68" s="16" t="inlineStr"/>
-      <c r="V68" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T68" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U68" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V68" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W68" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -8470,12 +9238,24 @@
       </c>
       <c r="S69" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T69" s="16" t="inlineStr"/>
-      <c r="U69" s="16" t="inlineStr"/>
-      <c r="V69" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T69" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U69" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V69" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W69" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -8583,12 +9363,24 @@
       </c>
       <c r="S70" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T70" s="16" t="inlineStr"/>
-      <c r="U70" s="16" t="inlineStr"/>
-      <c r="V70" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T70" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U70" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V70" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W70" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -8696,12 +9488,24 @@
       </c>
       <c r="S71" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T71" s="16" t="inlineStr"/>
-      <c r="U71" s="16" t="inlineStr"/>
-      <c r="V71" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T71" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U71" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V71" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W71" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -8809,12 +9613,24 @@
       </c>
       <c r="S72" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T72" s="16" t="inlineStr"/>
-      <c r="U72" s="16" t="inlineStr"/>
-      <c r="V72" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T72" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U72" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V72" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W72" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -8922,12 +9738,24 @@
       </c>
       <c r="S73" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T73" s="16" t="inlineStr"/>
-      <c r="U73" s="16" t="inlineStr"/>
-      <c r="V73" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T73" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U73" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V73" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W73" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -9035,12 +9863,24 @@
       </c>
       <c r="S74" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T74" s="16" t="inlineStr"/>
-      <c r="U74" s="16" t="inlineStr"/>
-      <c r="V74" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T74" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U74" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V74" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W74" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -9148,12 +9988,24 @@
       </c>
       <c r="S75" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T75" s="16" t="inlineStr"/>
-      <c r="U75" s="16" t="inlineStr"/>
-      <c r="V75" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T75" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U75" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V75" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W75" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -9261,12 +10113,24 @@
       </c>
       <c r="S76" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T76" s="16" t="inlineStr"/>
-      <c r="U76" s="16" t="inlineStr"/>
-      <c r="V76" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T76" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U76" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V76" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W76" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -9374,12 +10238,24 @@
       </c>
       <c r="S77" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T77" s="16" t="inlineStr"/>
-      <c r="U77" s="16" t="inlineStr"/>
-      <c r="V77" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T77" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U77" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V77" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W77" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -9487,12 +10363,24 @@
       </c>
       <c r="S78" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T78" s="16" t="inlineStr"/>
-      <c r="U78" s="16" t="inlineStr"/>
-      <c r="V78" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T78" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U78" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V78" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W78" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -9600,12 +10488,24 @@
       </c>
       <c r="S79" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T79" s="16" t="inlineStr"/>
-      <c r="U79" s="16" t="inlineStr"/>
-      <c r="V79" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T79" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U79" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V79" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W79" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -9713,12 +10613,24 @@
       </c>
       <c r="S80" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T80" s="16" t="inlineStr"/>
-      <c r="U80" s="16" t="inlineStr"/>
-      <c r="V80" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T80" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U80" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V80" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W80" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -9826,12 +10738,24 @@
       </c>
       <c r="S81" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T81" s="16" t="inlineStr"/>
-      <c r="U81" s="16" t="inlineStr"/>
-      <c r="V81" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T81" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U81" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V81" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W81" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -9939,12 +10863,24 @@
       </c>
       <c r="S82" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T82" s="16" t="inlineStr"/>
-      <c r="U82" s="16" t="inlineStr"/>
-      <c r="V82" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T82" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U82" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V82" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W82" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -10052,12 +10988,24 @@
       </c>
       <c r="S83" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T83" s="16" t="inlineStr"/>
-      <c r="U83" s="16" t="inlineStr"/>
-      <c r="V83" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T83" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U83" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V83" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W83" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -10165,12 +11113,24 @@
       </c>
       <c r="S84" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T84" s="16" t="inlineStr"/>
-      <c r="U84" s="16" t="inlineStr"/>
-      <c r="V84" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T84" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U84" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V84" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W84" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -10278,12 +11238,24 @@
       </c>
       <c r="S85" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T85" s="16" t="inlineStr"/>
-      <c r="U85" s="16" t="inlineStr"/>
-      <c r="V85" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T85" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U85" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V85" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W85" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -10391,12 +11363,24 @@
       </c>
       <c r="S86" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T86" s="16" t="inlineStr"/>
-      <c r="U86" s="16" t="inlineStr"/>
-      <c r="V86" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T86" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U86" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V86" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W86" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -10504,12 +11488,24 @@
       </c>
       <c r="S87" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T87" s="16" t="inlineStr"/>
-      <c r="U87" s="16" t="inlineStr"/>
-      <c r="V87" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T87" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U87" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V87" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W87" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -10617,12 +11613,24 @@
       </c>
       <c r="S88" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T88" s="16" t="inlineStr"/>
-      <c r="U88" s="16" t="inlineStr"/>
-      <c r="V88" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T88" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U88" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V88" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W88" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -10730,12 +11738,24 @@
       </c>
       <c r="S89" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T89" s="16" t="inlineStr"/>
-      <c r="U89" s="16" t="inlineStr"/>
-      <c r="V89" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T89" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U89" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V89" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W89" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -10843,12 +11863,24 @@
       </c>
       <c r="S90" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T90" s="16" t="inlineStr"/>
-      <c r="U90" s="16" t="inlineStr"/>
-      <c r="V90" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T90" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U90" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V90" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W90" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -10956,12 +11988,24 @@
       </c>
       <c r="S91" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T91" s="16" t="inlineStr"/>
-      <c r="U91" s="16" t="inlineStr"/>
-      <c r="V91" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T91" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U91" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V91" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W91" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -11069,12 +12113,24 @@
       </c>
       <c r="S92" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T92" s="16" t="inlineStr"/>
-      <c r="U92" s="16" t="inlineStr"/>
-      <c r="V92" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T92" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U92" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V92" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W92" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -11182,12 +12238,24 @@
       </c>
       <c r="S93" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T93" s="16" t="inlineStr"/>
-      <c r="U93" s="16" t="inlineStr"/>
-      <c r="V93" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T93" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U93" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V93" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W93" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -11295,12 +12363,24 @@
       </c>
       <c r="S94" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T94" s="16" t="inlineStr"/>
-      <c r="U94" s="16" t="inlineStr"/>
-      <c r="V94" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T94" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U94" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V94" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W94" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -11408,12 +12488,24 @@
       </c>
       <c r="S95" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T95" s="16" t="inlineStr"/>
-      <c r="U95" s="16" t="inlineStr"/>
-      <c r="V95" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T95" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U95" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V95" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W95" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -11521,12 +12613,24 @@
       </c>
       <c r="S96" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T96" s="16" t="inlineStr"/>
-      <c r="U96" s="16" t="inlineStr"/>
-      <c r="V96" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T96" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U96" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V96" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W96" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -11634,12 +12738,24 @@
       </c>
       <c r="S97" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T97" s="16" t="inlineStr"/>
-      <c r="U97" s="16" t="inlineStr"/>
-      <c r="V97" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T97" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U97" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V97" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W97" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -11747,12 +12863,24 @@
       </c>
       <c r="S98" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T98" s="16" t="inlineStr"/>
-      <c r="U98" s="16" t="inlineStr"/>
-      <c r="V98" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T98" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U98" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V98" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W98" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -11860,12 +12988,24 @@
       </c>
       <c r="S99" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T99" s="16" t="inlineStr"/>
-      <c r="U99" s="16" t="inlineStr"/>
-      <c r="V99" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T99" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U99" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V99" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W99" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -11973,12 +13113,24 @@
       </c>
       <c r="S100" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T100" s="16" t="inlineStr"/>
-      <c r="U100" s="16" t="inlineStr"/>
-      <c r="V100" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T100" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U100" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V100" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W100" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -12086,12 +13238,24 @@
       </c>
       <c r="S101" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T101" s="16" t="inlineStr"/>
-      <c r="U101" s="16" t="inlineStr"/>
-      <c r="V101" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T101" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U101" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V101" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W101" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -12199,12 +13363,24 @@
       </c>
       <c r="S102" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T102" s="16" t="inlineStr"/>
-      <c r="U102" s="16" t="inlineStr"/>
-      <c r="V102" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T102" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U102" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V102" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W102" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -12312,12 +13488,24 @@
       </c>
       <c r="S103" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T103" s="16" t="inlineStr"/>
-      <c r="U103" s="16" t="inlineStr"/>
-      <c r="V103" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T103" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U103" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V103" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W103" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -12425,12 +13613,24 @@
       </c>
       <c r="S104" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T104" s="16" t="inlineStr"/>
-      <c r="U104" s="16" t="inlineStr"/>
-      <c r="V104" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T104" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U104" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V104" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W104" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -12538,12 +13738,24 @@
       </c>
       <c r="S105" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T105" s="16" t="inlineStr"/>
-      <c r="U105" s="16" t="inlineStr"/>
-      <c r="V105" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T105" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U105" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V105" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W105" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -12651,12 +13863,24 @@
       </c>
       <c r="S106" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T106" s="16" t="inlineStr"/>
-      <c r="U106" s="16" t="inlineStr"/>
-      <c r="V106" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T106" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U106" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V106" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W106" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -12764,12 +13988,24 @@
       </c>
       <c r="S107" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T107" s="16" t="inlineStr"/>
-      <c r="U107" s="16" t="inlineStr"/>
-      <c r="V107" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T107" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U107" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V107" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W107" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -12877,12 +14113,24 @@
       </c>
       <c r="S108" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T108" s="16" t="inlineStr"/>
-      <c r="U108" s="16" t="inlineStr"/>
-      <c r="V108" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T108" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U108" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V108" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W108" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -12990,12 +14238,24 @@
       </c>
       <c r="S109" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T109" s="16" t="inlineStr"/>
-      <c r="U109" s="16" t="inlineStr"/>
-      <c r="V109" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T109" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U109" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V109" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W109" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -13103,12 +14363,24 @@
       </c>
       <c r="S110" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T110" s="16" t="inlineStr"/>
-      <c r="U110" s="16" t="inlineStr"/>
-      <c r="V110" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T110" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U110" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V110" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W110" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -13216,12 +14488,24 @@
       </c>
       <c r="S111" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T111" s="16" t="inlineStr"/>
-      <c r="U111" s="16" t="inlineStr"/>
-      <c r="V111" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T111" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U111" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V111" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W111" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -13329,12 +14613,24 @@
       </c>
       <c r="S112" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T112" s="16" t="inlineStr"/>
-      <c r="U112" s="16" t="inlineStr"/>
-      <c r="V112" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T112" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U112" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V112" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W112" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -13442,12 +14738,24 @@
       </c>
       <c r="S113" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T113" s="16" t="inlineStr"/>
-      <c r="U113" s="16" t="inlineStr"/>
-      <c r="V113" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T113" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U113" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V113" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W113" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -13555,12 +14863,24 @@
       </c>
       <c r="S114" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T114" s="16" t="inlineStr"/>
-      <c r="U114" s="16" t="inlineStr"/>
-      <c r="V114" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T114" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U114" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V114" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W114" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -13668,12 +14988,24 @@
       </c>
       <c r="S115" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T115" s="16" t="inlineStr"/>
-      <c r="U115" s="16" t="inlineStr"/>
-      <c r="V115" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T115" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U115" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V115" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W115" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -13781,12 +15113,24 @@
       </c>
       <c r="S116" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T116" s="16" t="inlineStr"/>
-      <c r="U116" s="16" t="inlineStr"/>
-      <c r="V116" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T116" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U116" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V116" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W116" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -13894,12 +15238,24 @@
       </c>
       <c r="S117" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T117" s="16" t="inlineStr"/>
-      <c r="U117" s="16" t="inlineStr"/>
-      <c r="V117" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T117" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U117" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V117" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W117" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -14007,12 +15363,24 @@
       </c>
       <c r="S118" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T118" s="16" t="inlineStr"/>
-      <c r="U118" s="16" t="inlineStr"/>
-      <c r="V118" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T118" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U118" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V118" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W118" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -14120,12 +15488,24 @@
       </c>
       <c r="S119" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T119" s="16" t="inlineStr"/>
-      <c r="U119" s="16" t="inlineStr"/>
-      <c r="V119" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T119" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U119" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V119" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W119" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -14233,12 +15613,24 @@
       </c>
       <c r="S120" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T120" s="16" t="inlineStr"/>
-      <c r="U120" s="16" t="inlineStr"/>
-      <c r="V120" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T120" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U120" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V120" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W120" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -14346,12 +15738,24 @@
       </c>
       <c r="S121" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T121" s="16" t="inlineStr"/>
-      <c r="U121" s="16" t="inlineStr"/>
-      <c r="V121" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T121" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U121" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V121" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W121" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -14459,12 +15863,24 @@
       </c>
       <c r="S122" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T122" s="16" t="inlineStr"/>
-      <c r="U122" s="16" t="inlineStr"/>
-      <c r="V122" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T122" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U122" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V122" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W122" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -14572,12 +15988,24 @@
       </c>
       <c r="S123" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T123" s="16" t="inlineStr"/>
-      <c r="U123" s="16" t="inlineStr"/>
-      <c r="V123" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T123" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U123" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V123" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W123" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -14685,12 +16113,24 @@
       </c>
       <c r="S124" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T124" s="16" t="inlineStr"/>
-      <c r="U124" s="16" t="inlineStr"/>
-      <c r="V124" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T124" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U124" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V124" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W124" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -14798,12 +16238,24 @@
       </c>
       <c r="S125" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T125" s="16" t="inlineStr"/>
-      <c r="U125" s="16" t="inlineStr"/>
-      <c r="V125" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T125" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U125" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V125" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W125" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -14911,12 +16363,24 @@
       </c>
       <c r="S126" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T126" s="16" t="inlineStr"/>
-      <c r="U126" s="16" t="inlineStr"/>
-      <c r="V126" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T126" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U126" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V126" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W126" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -15024,12 +16488,24 @@
       </c>
       <c r="S127" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T127" s="16" t="inlineStr"/>
-      <c r="U127" s="16" t="inlineStr"/>
-      <c r="V127" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T127" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U127" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V127" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W127" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -15137,12 +16613,24 @@
       </c>
       <c r="S128" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T128" s="16" t="inlineStr"/>
-      <c r="U128" s="16" t="inlineStr"/>
-      <c r="V128" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T128" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U128" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V128" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W128" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -15250,12 +16738,24 @@
       </c>
       <c r="S129" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T129" s="16" t="inlineStr"/>
-      <c r="U129" s="16" t="inlineStr"/>
-      <c r="V129" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T129" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U129" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V129" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W129" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -15363,12 +16863,24 @@
       </c>
       <c r="S130" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T130" s="16" t="inlineStr"/>
-      <c r="U130" s="16" t="inlineStr"/>
-      <c r="V130" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T130" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U130" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V130" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W130" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -15476,12 +16988,24 @@
       </c>
       <c r="S131" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T131" s="16" t="inlineStr"/>
-      <c r="U131" s="16" t="inlineStr"/>
-      <c r="V131" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T131" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U131" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V131" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W131" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -15589,12 +17113,24 @@
       </c>
       <c r="S132" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T132" s="16" t="inlineStr"/>
-      <c r="U132" s="16" t="inlineStr"/>
-      <c r="V132" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T132" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U132" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V132" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W132" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -15702,12 +17238,24 @@
       </c>
       <c r="S133" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T133" s="16" t="inlineStr"/>
-      <c r="U133" s="16" t="inlineStr"/>
-      <c r="V133" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T133" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U133" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V133" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W133" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -15815,12 +17363,24 @@
       </c>
       <c r="S134" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T134" s="16" t="inlineStr"/>
-      <c r="U134" s="16" t="inlineStr"/>
-      <c r="V134" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T134" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U134" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V134" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W134" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -16041,12 +17601,24 @@
       </c>
       <c r="S136" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T136" s="16" t="inlineStr"/>
-      <c r="U136" s="16" t="inlineStr"/>
-      <c r="V136" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T136" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U136" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V136" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W136" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -16154,12 +17726,24 @@
       </c>
       <c r="S137" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T137" s="16" t="inlineStr"/>
-      <c r="U137" s="16" t="inlineStr"/>
-      <c r="V137" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T137" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U137" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V137" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W137" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -16267,12 +17851,24 @@
       </c>
       <c r="S138" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T138" s="16" t="inlineStr"/>
-      <c r="U138" s="16" t="inlineStr"/>
-      <c r="V138" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T138" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U138" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V138" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W138" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -16380,12 +17976,24 @@
       </c>
       <c r="S139" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T139" s="16" t="inlineStr"/>
-      <c r="U139" s="16" t="inlineStr"/>
-      <c r="V139" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T139" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U139" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V139" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W139" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -16493,12 +18101,24 @@
       </c>
       <c r="S140" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T140" s="16" t="inlineStr"/>
-      <c r="U140" s="16" t="inlineStr"/>
-      <c r="V140" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T140" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U140" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V140" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W140" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -16606,12 +18226,24 @@
       </c>
       <c r="S141" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T141" s="16" t="inlineStr"/>
-      <c r="U141" s="16" t="inlineStr"/>
-      <c r="V141" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T141" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U141" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V141" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W141" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -16719,12 +18351,24 @@
       </c>
       <c r="S142" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T142" s="16" t="inlineStr"/>
-      <c r="U142" s="16" t="inlineStr"/>
-      <c r="V142" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T142" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U142" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V142" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W142" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -16832,12 +18476,24 @@
       </c>
       <c r="S143" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T143" s="16" t="inlineStr"/>
-      <c r="U143" s="16" t="inlineStr"/>
-      <c r="V143" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T143" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U143" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V143" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W143" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>
@@ -16945,12 +18601,24 @@
       </c>
       <c r="S144" s="16" t="inlineStr">
         <is>
-          <t>NOT_RUN</t>
-        </is>
-      </c>
-      <c r="T144" s="16" t="inlineStr"/>
-      <c r="U144" s="16" t="inlineStr"/>
-      <c r="V144" s="16" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T144" s="16" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U144" s="16" t="inlineStr">
+        <is>
+          <t>39c48ee</t>
+        </is>
+      </c>
+      <c r="V144" s="16" t="inlineStr">
+        <is>
+          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+        </is>
+      </c>
       <c r="W144" s="16" t="inlineStr">
         <is>
           <t>NOT_RUN</t>

</xml_diff>

<commit_message>
fix: out_dir double-tb bug; gap_report at IP root; COV stubs generated
- config.py: [output] dir now sets out_dir=toml_dir (IP root) instead
  of _resolve(dir_value). Since D-032, generate_uvm_tb() always appends
  /tb/ itself; resolving dir="tb" to IP_root/tb then adding /tb produced
  the tb/tb/ double nesting.
- test_config.py: updated test_config_load_reads_output_section to
  assert out_dir == FIXTURES_DIR (IP root) per new semantics.
- Deleted stray ip/buffered_axi_lite_uart/tb/tb/ (untracked, from
  buggy no---out run); deleted wrong-location tb/gap_report.json.
- gap_report.json now written to IP root (ip/buffered_axi_lite_uart/).
- VPR write-back confirmed: 139 rows updated, gap_report.json at IP root.
- 250 tests pass.

Author: S. Belvin, BelTech Systems LLC

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ip/buffered_axi_lite_uart/buffered_axi_lite_uart_vplan.xlsx
+++ b/ip/buffered_axi_lite_uart/buffered_axi_lite_uart_vplan.xlsx
@@ -1143,7 +1143,7 @@
       </c>
       <c r="U4" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V4" s="16" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="U5" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V5" s="16" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="U7" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V7" s="16" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="U8" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V8" s="16" t="inlineStr">
@@ -1756,7 +1756,7 @@
       </c>
       <c r="U9" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V9" s="16" t="inlineStr">
@@ -1881,7 +1881,7 @@
       </c>
       <c r="U10" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V10" s="16" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="U11" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V11" s="16" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="U12" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V12" s="16" t="inlineStr">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="U13" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V13" s="16" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="U14" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V14" s="16" t="inlineStr">
@@ -2506,7 +2506,7 @@
       </c>
       <c r="U15" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V15" s="16" t="inlineStr">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="U16" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V16" s="16" t="inlineStr">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="U17" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V17" s="16" t="inlineStr">
@@ -2881,7 +2881,7 @@
       </c>
       <c r="U18" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V18" s="16" t="inlineStr">
@@ -3006,7 +3006,7 @@
       </c>
       <c r="U19" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V19" s="16" t="inlineStr">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="U20" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V20" s="16" t="inlineStr">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="U21" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V21" s="16" t="inlineStr">
@@ -3381,7 +3381,7 @@
       </c>
       <c r="U22" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V22" s="16" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="U23" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V23" s="16" t="inlineStr">
@@ -3631,7 +3631,7 @@
       </c>
       <c r="U24" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V24" s="16" t="inlineStr">
@@ -3756,7 +3756,7 @@
       </c>
       <c r="U25" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V25" s="16" t="inlineStr">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="U26" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V26" s="16" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="U27" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V27" s="16" t="inlineStr">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="U28" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V28" s="16" t="inlineStr">
@@ -4256,7 +4256,7 @@
       </c>
       <c r="U29" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V29" s="16" t="inlineStr">
@@ -4381,7 +4381,7 @@
       </c>
       <c r="U30" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V30" s="16" t="inlineStr">
@@ -4506,7 +4506,7 @@
       </c>
       <c r="U31" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V31" s="16" t="inlineStr">
@@ -4631,7 +4631,7 @@
       </c>
       <c r="U32" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V32" s="16" t="inlineStr">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="U33" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V33" s="16" t="inlineStr">
@@ -4881,7 +4881,7 @@
       </c>
       <c r="U34" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V34" s="16" t="inlineStr">
@@ -5006,7 +5006,7 @@
       </c>
       <c r="U35" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V35" s="16" t="inlineStr">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="U36" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V36" s="16" t="inlineStr">
@@ -5248,7 +5248,7 @@
       </c>
       <c r="U37" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V37" s="16" t="inlineStr">
@@ -5373,7 +5373,7 @@
       </c>
       <c r="U38" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V38" s="16" t="inlineStr">
@@ -5498,7 +5498,7 @@
       </c>
       <c r="U39" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V39" s="16" t="inlineStr">
@@ -5623,7 +5623,7 @@
       </c>
       <c r="U40" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V40" s="16" t="inlineStr">
@@ -5748,7 +5748,7 @@
       </c>
       <c r="U41" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V41" s="16" t="inlineStr">
@@ -5873,7 +5873,7 @@
       </c>
       <c r="U42" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V42" s="16" t="inlineStr">
@@ -5998,7 +5998,7 @@
       </c>
       <c r="U43" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V43" s="16" t="inlineStr">
@@ -6123,7 +6123,7 @@
       </c>
       <c r="U44" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V44" s="16" t="inlineStr">
@@ -6248,7 +6248,7 @@
       </c>
       <c r="U45" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V45" s="16" t="inlineStr">
@@ -6373,7 +6373,7 @@
       </c>
       <c r="U46" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V46" s="16" t="inlineStr">
@@ -6498,7 +6498,7 @@
       </c>
       <c r="U47" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V47" s="16" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="U48" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V48" s="16" t="inlineStr">
@@ -6748,7 +6748,7 @@
       </c>
       <c r="U49" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V49" s="16" t="inlineStr">
@@ -6873,7 +6873,7 @@
       </c>
       <c r="U50" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V50" s="16" t="inlineStr">
@@ -6998,7 +6998,7 @@
       </c>
       <c r="U51" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V51" s="16" t="inlineStr">
@@ -7123,7 +7123,7 @@
       </c>
       <c r="U52" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V52" s="16" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="U53" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V53" s="16" t="inlineStr">
@@ -7373,7 +7373,7 @@
       </c>
       <c r="U54" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V54" s="16" t="inlineStr">
@@ -7498,7 +7498,7 @@
       </c>
       <c r="U55" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V55" s="16" t="inlineStr">
@@ -7623,7 +7623,7 @@
       </c>
       <c r="U56" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V56" s="16" t="inlineStr">
@@ -7748,7 +7748,7 @@
       </c>
       <c r="U57" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V57" s="16" t="inlineStr">
@@ -7873,7 +7873,7 @@
       </c>
       <c r="U58" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V58" s="16" t="inlineStr">
@@ -7998,7 +7998,7 @@
       </c>
       <c r="U59" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V59" s="16" t="inlineStr">
@@ -8123,7 +8123,7 @@
       </c>
       <c r="U60" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V60" s="16" t="inlineStr">
@@ -8248,7 +8248,7 @@
       </c>
       <c r="U61" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V61" s="16" t="inlineStr">
@@ -8373,7 +8373,7 @@
       </c>
       <c r="U62" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V62" s="16" t="inlineStr">
@@ -8498,7 +8498,7 @@
       </c>
       <c r="U63" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V63" s="16" t="inlineStr">
@@ -8623,7 +8623,7 @@
       </c>
       <c r="U64" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V64" s="16" t="inlineStr">
@@ -8748,7 +8748,7 @@
       </c>
       <c r="U65" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V65" s="16" t="inlineStr">
@@ -8873,7 +8873,7 @@
       </c>
       <c r="U66" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V66" s="16" t="inlineStr">
@@ -8998,7 +8998,7 @@
       </c>
       <c r="U67" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V67" s="16" t="inlineStr">
@@ -9123,7 +9123,7 @@
       </c>
       <c r="U68" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V68" s="16" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="U69" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V69" s="16" t="inlineStr">
@@ -9373,7 +9373,7 @@
       </c>
       <c r="U70" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V70" s="16" t="inlineStr">
@@ -9498,7 +9498,7 @@
       </c>
       <c r="U71" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V71" s="16" t="inlineStr">
@@ -9623,7 +9623,7 @@
       </c>
       <c r="U72" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V72" s="16" t="inlineStr">
@@ -9748,7 +9748,7 @@
       </c>
       <c r="U73" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V73" s="16" t="inlineStr">
@@ -9873,7 +9873,7 @@
       </c>
       <c r="U74" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V74" s="16" t="inlineStr">
@@ -9998,7 +9998,7 @@
       </c>
       <c r="U75" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V75" s="16" t="inlineStr">
@@ -10123,7 +10123,7 @@
       </c>
       <c r="U76" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V76" s="16" t="inlineStr">
@@ -10248,7 +10248,7 @@
       </c>
       <c r="U77" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V77" s="16" t="inlineStr">
@@ -10373,7 +10373,7 @@
       </c>
       <c r="U78" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V78" s="16" t="inlineStr">
@@ -10498,7 +10498,7 @@
       </c>
       <c r="U79" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V79" s="16" t="inlineStr">
@@ -10623,7 +10623,7 @@
       </c>
       <c r="U80" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V80" s="16" t="inlineStr">
@@ -10748,7 +10748,7 @@
       </c>
       <c r="U81" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V81" s="16" t="inlineStr">
@@ -10873,7 +10873,7 @@
       </c>
       <c r="U82" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V82" s="16" t="inlineStr">
@@ -10998,7 +10998,7 @@
       </c>
       <c r="U83" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V83" s="16" t="inlineStr">
@@ -11123,7 +11123,7 @@
       </c>
       <c r="U84" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V84" s="16" t="inlineStr">
@@ -11248,7 +11248,7 @@
       </c>
       <c r="U85" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V85" s="16" t="inlineStr">
@@ -11373,7 +11373,7 @@
       </c>
       <c r="U86" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V86" s="16" t="inlineStr">
@@ -11498,7 +11498,7 @@
       </c>
       <c r="U87" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V87" s="16" t="inlineStr">
@@ -11623,7 +11623,7 @@
       </c>
       <c r="U88" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V88" s="16" t="inlineStr">
@@ -11748,7 +11748,7 @@
       </c>
       <c r="U89" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V89" s="16" t="inlineStr">
@@ -11873,7 +11873,7 @@
       </c>
       <c r="U90" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V90" s="16" t="inlineStr">
@@ -11998,7 +11998,7 @@
       </c>
       <c r="U91" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V91" s="16" t="inlineStr">
@@ -12123,7 +12123,7 @@
       </c>
       <c r="U92" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V92" s="16" t="inlineStr">
@@ -12248,7 +12248,7 @@
       </c>
       <c r="U93" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V93" s="16" t="inlineStr">
@@ -12373,7 +12373,7 @@
       </c>
       <c r="U94" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V94" s="16" t="inlineStr">
@@ -12498,7 +12498,7 @@
       </c>
       <c r="U95" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V95" s="16" t="inlineStr">
@@ -12623,7 +12623,7 @@
       </c>
       <c r="U96" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V96" s="16" t="inlineStr">
@@ -12748,7 +12748,7 @@
       </c>
       <c r="U97" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V97" s="16" t="inlineStr">
@@ -12873,7 +12873,7 @@
       </c>
       <c r="U98" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V98" s="16" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="U99" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V99" s="16" t="inlineStr">
@@ -13123,7 +13123,7 @@
       </c>
       <c r="U100" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V100" s="16" t="inlineStr">
@@ -13248,7 +13248,7 @@
       </c>
       <c r="U101" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V101" s="16" t="inlineStr">
@@ -13373,7 +13373,7 @@
       </c>
       <c r="U102" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V102" s="16" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="U103" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V103" s="16" t="inlineStr">
@@ -13623,7 +13623,7 @@
       </c>
       <c r="U104" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V104" s="16" t="inlineStr">
@@ -13748,7 +13748,7 @@
       </c>
       <c r="U105" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V105" s="16" t="inlineStr">
@@ -13873,7 +13873,7 @@
       </c>
       <c r="U106" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V106" s="16" t="inlineStr">
@@ -13998,7 +13998,7 @@
       </c>
       <c r="U107" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V107" s="16" t="inlineStr">
@@ -14123,7 +14123,7 @@
       </c>
       <c r="U108" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V108" s="16" t="inlineStr">
@@ -14248,7 +14248,7 @@
       </c>
       <c r="U109" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V109" s="16" t="inlineStr">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="U110" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V110" s="16" t="inlineStr">
@@ -14498,7 +14498,7 @@
       </c>
       <c r="U111" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V111" s="16" t="inlineStr">
@@ -14623,7 +14623,7 @@
       </c>
       <c r="U112" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V112" s="16" t="inlineStr">
@@ -14748,7 +14748,7 @@
       </c>
       <c r="U113" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V113" s="16" t="inlineStr">
@@ -14873,7 +14873,7 @@
       </c>
       <c r="U114" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V114" s="16" t="inlineStr">
@@ -14998,7 +14998,7 @@
       </c>
       <c r="U115" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V115" s="16" t="inlineStr">
@@ -15123,7 +15123,7 @@
       </c>
       <c r="U116" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V116" s="16" t="inlineStr">
@@ -15248,7 +15248,7 @@
       </c>
       <c r="U117" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V117" s="16" t="inlineStr">
@@ -15373,7 +15373,7 @@
       </c>
       <c r="U118" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V118" s="16" t="inlineStr">
@@ -15498,7 +15498,7 @@
       </c>
       <c r="U119" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V119" s="16" t="inlineStr">
@@ -15623,7 +15623,7 @@
       </c>
       <c r="U120" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V120" s="16" t="inlineStr">
@@ -15748,7 +15748,7 @@
       </c>
       <c r="U121" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V121" s="16" t="inlineStr">
@@ -15873,7 +15873,7 @@
       </c>
       <c r="U122" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V122" s="16" t="inlineStr">
@@ -15998,7 +15998,7 @@
       </c>
       <c r="U123" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V123" s="16" t="inlineStr">
@@ -16123,7 +16123,7 @@
       </c>
       <c r="U124" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V124" s="16" t="inlineStr">
@@ -16248,7 +16248,7 @@
       </c>
       <c r="U125" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V125" s="16" t="inlineStr">
@@ -16373,7 +16373,7 @@
       </c>
       <c r="U126" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V126" s="16" t="inlineStr">
@@ -16498,7 +16498,7 @@
       </c>
       <c r="U127" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V127" s="16" t="inlineStr">
@@ -16623,7 +16623,7 @@
       </c>
       <c r="U128" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V128" s="16" t="inlineStr">
@@ -16748,7 +16748,7 @@
       </c>
       <c r="U129" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V129" s="16" t="inlineStr">
@@ -16873,7 +16873,7 @@
       </c>
       <c r="U130" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V130" s="16" t="inlineStr">
@@ -16998,7 +16998,7 @@
       </c>
       <c r="U131" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V131" s="16" t="inlineStr">
@@ -17123,7 +17123,7 @@
       </c>
       <c r="U132" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V132" s="16" t="inlineStr">
@@ -17248,7 +17248,7 @@
       </c>
       <c r="U133" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V133" s="16" t="inlineStr">
@@ -17373,7 +17373,7 @@
       </c>
       <c r="U134" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V134" s="16" t="inlineStr">
@@ -17611,7 +17611,7 @@
       </c>
       <c r="U136" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V136" s="16" t="inlineStr">
@@ -17736,7 +17736,7 @@
       </c>
       <c r="U137" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V137" s="16" t="inlineStr">
@@ -17861,7 +17861,7 @@
       </c>
       <c r="U138" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V138" s="16" t="inlineStr">
@@ -17986,7 +17986,7 @@
       </c>
       <c r="U139" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V139" s="16" t="inlineStr">
@@ -18111,7 +18111,7 @@
       </c>
       <c r="U140" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V140" s="16" t="inlineStr">
@@ -18236,7 +18236,7 @@
       </c>
       <c r="U141" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V141" s="16" t="inlineStr">
@@ -18361,7 +18361,7 @@
       </c>
       <c r="U142" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V142" s="16" t="inlineStr">
@@ -18486,7 +18486,7 @@
       </c>
       <c r="U143" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V143" s="16" t="inlineStr">
@@ -18611,7 +18611,7 @@
       </c>
       <c r="U144" s="16" t="inlineStr">
         <is>
-          <t>39c48ee</t>
+          <t>0148f1e</t>
         </is>
       </c>
       <c r="V144" s="16" t="inlineStr">

</xml_diff>

<commit_message>
D-034 Step 4: Phase 1 BALU sequence body generation from VSL
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ip/buffered_axi_lite_uart/buffered_axi_lite_uart_vplan.xlsx
+++ b/ip/buffered_axi_lite_uart/buffered_axi_lite_uart_vplan.xlsx
@@ -18830,10 +18830,14 @@
       <c r="I3" s="16" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr"/>
+          <t>PHASE_1</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>WRITE,addr=0x08,data=0x000010D6;WAIT,cycles=256;POLL,addr=0x0C,mask=0x01,expect=0x01,timeout=1000</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
@@ -18882,7 +18886,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -18931,7 +18934,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
@@ -18980,7 +18982,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
@@ -19029,7 +19030,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
@@ -19078,7 +19078,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
@@ -19127,7 +19126,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
@@ -19176,7 +19174,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
@@ -19225,7 +19222,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
@@ -19271,10 +19267,14 @@
       <c r="I12" s="16" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr"/>
+          <t>PHASE_1</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>WRITE,addr=0x00,data=0x00000001;READ,addr=0x0C,expect=0x00</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
@@ -19323,7 +19323,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="16" t="inlineStr">
@@ -19372,7 +19371,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
@@ -19425,7 +19423,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
@@ -19475,10 +19472,14 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr"/>
+          <t>PHASE_1</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>WRITE,addr=0x2C,data=0x00000001;READ,addr=0x2C,expect=0x00000001</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="16" t="inlineStr">
@@ -19527,7 +19528,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
@@ -19576,7 +19576,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="16" t="inlineStr">
@@ -19625,7 +19624,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="16" t="inlineStr">
@@ -19674,7 +19672,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="16" t="inlineStr">
@@ -19723,7 +19720,6 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
D-034 Step 5: BALU regression results + Grafana D-034 Phase 1 panel
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ip/buffered_axi_lite_uart/buffered_axi_lite_uart_vplan.xlsx
+++ b/ip/buffered_axi_lite_uart/buffered_axi_lite_uart_vplan.xlsx
@@ -18819,7 +18819,7 @@
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>WRITTEN</t>
         </is>
       </c>
       <c r="H3" s="16" t="inlineStr">
@@ -19256,7 +19256,7 @@
       </c>
       <c r="G12" s="16" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>WRITTEN</t>
         </is>
       </c>
       <c r="H12" s="16" t="inlineStr">
@@ -19457,7 +19457,7 @@
       </c>
       <c r="G16" s="16" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>WRITTEN</t>
         </is>
       </c>
       <c r="H16" s="16" t="inlineStr">

</xml_diff>

<commit_message>
D-034 Step 5b: batch VSL authoring for 16 BALU goals, 100% Phase 1 coverage
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ip/buffered_axi_lite_uart/buffered_axi_lite_uart_vplan.xlsx
+++ b/ip/buffered_axi_lite_uart/buffered_axi_lite_uart_vplan.xlsx
@@ -18872,7 +18872,7 @@
       </c>
       <c r="G4" s="16" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>WRITTEN</t>
         </is>
       </c>
       <c r="H4" s="16" t="inlineStr">
@@ -18883,7 +18883,12 @@
       <c r="I4" s="16" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PHASE_1</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>WRITE,addr=0x34,data=0x01;WRITE,addr=0x24,data=0x01;WRITE,addr=0x00,data=0x03;WRITE,addr=0x0C,data=0x41;POLL,addr=0x04,mask=0x02,expect=0x02,timeout=1000;READ,addr=0x10,expect=0x41</t>
         </is>
       </c>
     </row>
@@ -18920,7 +18925,7 @@
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>WRITTEN</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr">
@@ -18931,7 +18936,12 @@
       <c r="I5" s="16" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PHASE_1</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>WRITE,addr=0x34,data=0x01;WRITE,addr=0x28,data=0x08;WRITE,addr=0x00,data=0x03;WRITE,addr=0x0C,data=0x55;POLL,addr=0x04,mask=0x02,expect=0x02,timeout=1000;READ,addr=0x10,expect=0x55</t>
         </is>
       </c>
     </row>
@@ -18968,7 +18978,7 @@
       </c>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>WRITTEN</t>
         </is>
       </c>
       <c r="H6" s="16" t="inlineStr">
@@ -18979,7 +18989,12 @@
       <c r="I6" s="16" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PHASE_1</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>WRITE,addr=0x34,data=0x01;WRITE,addr=0x00,data=0x03;WRITE,addr=0x0C,data=0xAA;POLL,addr=0x04,mask=0x02,expect=0x02,timeout=1000;READ,addr=0x18</t>
         </is>
       </c>
     </row>
@@ -19016,7 +19031,7 @@
       </c>
       <c r="G7" s="16" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>WRITTEN</t>
         </is>
       </c>
       <c r="H7" s="16" t="inlineStr">
@@ -19027,7 +19042,12 @@
       <c r="I7" s="16" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PHASE_1</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>WRITE,addr=0x00,data=0x01;WRITE,addr=0x0C,data=0xAA;WRITE,addr=0x0C,data=0x55;WRITE,addr=0x0C,data=0xFF;READ,addr=0x14</t>
         </is>
       </c>
     </row>
@@ -19064,7 +19084,7 @@
       </c>
       <c r="G8" s="16" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>WRITTEN</t>
         </is>
       </c>
       <c r="H8" s="16" t="inlineStr">
@@ -19075,7 +19095,12 @@
       <c r="I8" s="16" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PHASE_1</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>WRITE,addr=0x30,data=0x0001;READ,addr=0x30,expect=0x0001;WRITE,addr=0x30,data=0xFFFF;READ,addr=0x30,expect=0xFFFF</t>
         </is>
       </c>
     </row>
@@ -19112,7 +19137,7 @@
       </c>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>WRITTEN</t>
         </is>
       </c>
       <c r="H9" s="16" t="inlineStr">
@@ -19123,7 +19148,12 @@
       <c r="I9" s="16" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PHASE_1</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>WRITE,addr=0x1C,data=0x01;WRITE,addr=0x00,data=0x01;POLL,addr=0x20,mask=0x01,expect=0x01,timeout=100;WRITE,addr=0x20,data=0x01;READ,addr=0x20,expect=0x00</t>
         </is>
       </c>
     </row>
@@ -19160,7 +19190,7 @@
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>WRITTEN</t>
         </is>
       </c>
       <c r="H10" s="16" t="inlineStr">
@@ -19171,7 +19201,12 @@
       <c r="I10" s="16" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PHASE_1</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>WRITE,addr=0x34,data=0x01;WRITE,addr=0x1C,data=0x48;WRITE,addr=0x00,data=0x03;WRITE,addr=0x0C,data=0xFF;POLL,addr=0x04,mask=0x08,expect=0x08,timeout=2000;READ,addr=0x20</t>
         </is>
       </c>
     </row>
@@ -19208,7 +19243,7 @@
       </c>
       <c r="G11" s="16" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>WRITTEN</t>
         </is>
       </c>
       <c r="H11" s="16" t="inlineStr">
@@ -19219,7 +19254,12 @@
       <c r="I11" s="16" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PHASE_1</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>WRITE,addr=0x30,data=0x0010;WRITE,addr=0x1C,data=0x12;WRITE,addr=0x34,data=0x01;WRITE,addr=0x00,data=0x03;WRITE,addr=0x0C,data=0xAB;POLL,addr=0x20,mask=0x10,expect=0x10,timeout=2000</t>
         </is>
       </c>
     </row>
@@ -19309,7 +19349,7 @@
       </c>
       <c r="G13" s="16" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>WRITTEN</t>
         </is>
       </c>
       <c r="H13" s="16" t="inlineStr">
@@ -19320,7 +19360,12 @@
       <c r="I13" s="16" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PHASE_1</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>WRITE,addr=0x00,data=0x03;READ,addr=0x00,expect=0x03;READ,addr=0x04;READ,addr=0x08</t>
         </is>
       </c>
     </row>
@@ -19357,7 +19402,7 @@
       </c>
       <c r="G14" s="16" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>WRITTEN</t>
         </is>
       </c>
       <c r="H14" s="16" t="inlineStr">
@@ -19368,7 +19413,12 @@
       <c r="I14" s="16" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PHASE_1</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>WRITE,addr=0x2C,data=0xA5A5;READ,addr=0x2C,expect=0xA5A5;WRITE,addr=0x2C,data=0x5A5A;READ,addr=0x2C,expect=0x5A5A</t>
         </is>
       </c>
     </row>
@@ -19405,7 +19455,7 @@
       </c>
       <c r="G15" s="16" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>WRITTEN</t>
         </is>
       </c>
       <c r="H15" s="16" t="inlineStr">
@@ -19420,7 +19470,12 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PHASE_1</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>WRITE,addr=0x08,data=0x000010D6;WRITE,addr=0x00,data=0x03;WRITE,addr=0x08,data=0x00000001;READ,addr=0x08</t>
         </is>
       </c>
     </row>
@@ -19514,7 +19569,7 @@
       </c>
       <c r="G17" s="16" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>WRITTEN</t>
         </is>
       </c>
       <c r="H17" s="16" t="inlineStr">
@@ -19525,7 +19580,12 @@
       <c r="I17" s="16" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PHASE_1</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>WRITE,addr=0x00,data=0x80;WAIT,cycles=10;READ,addr=0x00;READ,addr=0x04,expect=0x01;READ,addr=0x08</t>
         </is>
       </c>
     </row>
@@ -19562,7 +19622,7 @@
       </c>
       <c r="G18" s="16" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>WRITTEN</t>
         </is>
       </c>
       <c r="H18" s="16" t="inlineStr">
@@ -19573,7 +19633,12 @@
       <c r="I18" s="16" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PHASE_1</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>WRITE,addr=0x00,data=0x01;READ,addr=0x04;WRITE,addr=0x00,data=0x02;READ,addr=0x04;WRITE,addr=0x00,data=0x03;READ,addr=0x04</t>
         </is>
       </c>
     </row>
@@ -19610,7 +19675,7 @@
       </c>
       <c r="G19" s="16" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>WRITTEN</t>
         </is>
       </c>
       <c r="H19" s="16" t="inlineStr">
@@ -19621,7 +19686,12 @@
       <c r="I19" s="16" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PHASE_1</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>WRITE,addr=0x28,data=0x08;READ,addr=0x28,expect=0x08;WRITE,addr=0x34,data=0x01;WRITE,addr=0x00,data=0x03;WRITE,addr=0x0C,data=0xA5</t>
         </is>
       </c>
     </row>
@@ -19658,7 +19728,7 @@
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>WRITTEN</t>
         </is>
       </c>
       <c r="H20" s="16" t="inlineStr">
@@ -19669,7 +19739,12 @@
       <c r="I20" s="16" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PHASE_1</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>READ,addr=0x04;WRITE,addr=0x04,data=0xFF;READ,addr=0x04;READ,addr=0x14;WRITE,addr=0x14,data=0xFF;READ,addr=0x14</t>
         </is>
       </c>
     </row>
@@ -19706,7 +19781,7 @@
       </c>
       <c r="G21" s="16" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>WRITTEN</t>
         </is>
       </c>
       <c r="H21" s="16" t="inlineStr">
@@ -19717,7 +19792,12 @@
       <c r="I21" s="16" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PHASE_1</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>WRITE,addr=0x1C,data=0x06;WRITE,addr=0x28,data=0x08;WRITE,addr=0x34,data=0x01;WRITE,addr=0x00,data=0x03;WRITE,addr=0x0C,data=0xAB;POLL,addr=0x20,mask=0x06,expect=0x02,timeout=1000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
RAL Session 3: post-regression results — PASS 0E/0F, coverage 94.8%
Regression 5 results (commit 19eec7a, RTL Fix 13):
  UVM_ERROR=0  UVM_FATAL=0  UVM_WARNING=3  coverage=94.8%

VPR write-back: 139 rows updated to PASS.
gap_report.json regenerated for Streamlit/Grafana dashboard.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ip/buffered_axi_lite_uart/buffered_axi_lite_uart_vplan.xlsx
+++ b/ip/buffered_axi_lite_uart/buffered_axi_lite_uart_vplan.xlsx
@@ -1060,17 +1060,17 @@
       </c>
       <c r="T4" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1185,17 +1185,17 @@
       </c>
       <c r="T5" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U5" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V5" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W5" s="5" t="inlineStr">
@@ -1423,17 +1423,17 @@
       </c>
       <c r="T7" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U7" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V7" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W7" s="5" t="inlineStr">
@@ -1548,17 +1548,17 @@
       </c>
       <c r="T8" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1673,17 +1673,17 @@
       </c>
       <c r="T9" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U9" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V9" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W9" s="5" t="inlineStr">
@@ -1798,17 +1798,17 @@
       </c>
       <c r="T10" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1923,17 +1923,17 @@
       </c>
       <c r="T11" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U11" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V11" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W11" s="5" t="inlineStr">
@@ -2048,17 +2048,17 @@
       </c>
       <c r="T12" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
@@ -2173,17 +2173,17 @@
       </c>
       <c r="T13" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U13" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V13" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W13" s="5" t="inlineStr">
@@ -2298,17 +2298,17 @@
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V14" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W14" s="5" t="inlineStr">
@@ -2423,17 +2423,17 @@
       </c>
       <c r="T15" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U15" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V15" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W15" s="5" t="inlineStr">
@@ -2548,17 +2548,17 @@
       </c>
       <c r="T16" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V16" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W16" s="5" t="inlineStr">
@@ -2673,17 +2673,17 @@
       </c>
       <c r="T17" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U17" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V17" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W17" s="5" t="inlineStr">
@@ -2798,17 +2798,17 @@
       </c>
       <c r="T18" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V18" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W18" s="5" t="inlineStr">
@@ -2923,17 +2923,17 @@
       </c>
       <c r="T19" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U19" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V19" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W19" s="5" t="inlineStr">
@@ -3048,17 +3048,17 @@
       </c>
       <c r="T20" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V20" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W20" s="5" t="inlineStr">
@@ -3173,17 +3173,17 @@
       </c>
       <c r="T21" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U21" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V21" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W21" s="5" t="inlineStr">
@@ -3298,17 +3298,17 @@
       </c>
       <c r="T22" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U22" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V22" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W22" s="5" t="inlineStr">
@@ -3423,17 +3423,17 @@
       </c>
       <c r="T23" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U23" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V23" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W23" s="5" t="inlineStr">
@@ -3548,17 +3548,17 @@
       </c>
       <c r="T24" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U24" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V24" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W24" s="5" t="inlineStr">
@@ -3673,17 +3673,17 @@
       </c>
       <c r="T25" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U25" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V25" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W25" s="5" t="inlineStr">
@@ -3798,17 +3798,17 @@
       </c>
       <c r="T26" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U26" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V26" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W26" s="5" t="inlineStr">
@@ -3923,17 +3923,17 @@
       </c>
       <c r="T27" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U27" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V27" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W27" s="5" t="inlineStr">
@@ -4048,17 +4048,17 @@
       </c>
       <c r="T28" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U28" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V28" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W28" s="5" t="inlineStr">
@@ -4173,17 +4173,17 @@
       </c>
       <c r="T29" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U29" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V29" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W29" s="5" t="inlineStr">
@@ -4298,17 +4298,17 @@
       </c>
       <c r="T30" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U30" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V30" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W30" s="5" t="inlineStr">
@@ -4423,17 +4423,17 @@
       </c>
       <c r="T31" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U31" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V31" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W31" s="5" t="inlineStr">
@@ -4548,17 +4548,17 @@
       </c>
       <c r="T32" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U32" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V32" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W32" s="5" t="inlineStr">
@@ -4673,17 +4673,17 @@
       </c>
       <c r="T33" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U33" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V33" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W33" s="5" t="inlineStr">
@@ -4798,17 +4798,17 @@
       </c>
       <c r="T34" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U34" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V34" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W34" s="5" t="inlineStr">
@@ -4923,17 +4923,17 @@
       </c>
       <c r="T35" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U35" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V35" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W35" s="5" t="inlineStr">
@@ -5040,17 +5040,17 @@
       </c>
       <c r="T36" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U36" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V36" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W36" s="5" t="inlineStr">
@@ -5165,17 +5165,17 @@
       </c>
       <c r="T37" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U37" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V37" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W37" s="5" t="inlineStr">
@@ -5290,17 +5290,17 @@
       </c>
       <c r="T38" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U38" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V38" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W38" s="5" t="inlineStr">
@@ -5415,17 +5415,17 @@
       </c>
       <c r="T39" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U39" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V39" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W39" s="5" t="inlineStr">
@@ -5540,17 +5540,17 @@
       </c>
       <c r="T40" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U40" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V40" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W40" s="5" t="inlineStr">
@@ -5665,17 +5665,17 @@
       </c>
       <c r="T41" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U41" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V41" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W41" s="5" t="inlineStr">
@@ -5790,17 +5790,17 @@
       </c>
       <c r="T42" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U42" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V42" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W42" s="5" t="inlineStr">
@@ -5915,17 +5915,17 @@
       </c>
       <c r="T43" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U43" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V43" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W43" s="5" t="inlineStr">
@@ -6040,17 +6040,17 @@
       </c>
       <c r="T44" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U44" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V44" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W44" s="5" t="inlineStr">
@@ -6165,17 +6165,17 @@
       </c>
       <c r="T45" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U45" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V45" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W45" s="5" t="inlineStr">
@@ -6290,17 +6290,17 @@
       </c>
       <c r="T46" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U46" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V46" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W46" s="5" t="inlineStr">
@@ -6415,17 +6415,17 @@
       </c>
       <c r="T47" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U47" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V47" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W47" s="5" t="inlineStr">
@@ -6540,17 +6540,17 @@
       </c>
       <c r="T48" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U48" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V48" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W48" s="5" t="inlineStr">
@@ -6665,17 +6665,17 @@
       </c>
       <c r="T49" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U49" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V49" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W49" s="5" t="inlineStr">
@@ -6790,17 +6790,17 @@
       </c>
       <c r="T50" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U50" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V50" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W50" s="5" t="inlineStr">
@@ -6915,17 +6915,17 @@
       </c>
       <c r="T51" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U51" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V51" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W51" s="5" t="inlineStr">
@@ -7040,17 +7040,17 @@
       </c>
       <c r="T52" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U52" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V52" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W52" s="5" t="inlineStr">
@@ -7165,17 +7165,17 @@
       </c>
       <c r="T53" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U53" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V53" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W53" s="5" t="inlineStr">
@@ -7290,17 +7290,17 @@
       </c>
       <c r="T54" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U54" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V54" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W54" s="5" t="inlineStr">
@@ -7415,17 +7415,17 @@
       </c>
       <c r="T55" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U55" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V55" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W55" s="5" t="inlineStr">
@@ -7540,17 +7540,17 @@
       </c>
       <c r="T56" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U56" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V56" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W56" s="5" t="inlineStr">
@@ -7665,17 +7665,17 @@
       </c>
       <c r="T57" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U57" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V57" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W57" s="5" t="inlineStr">
@@ -7790,17 +7790,17 @@
       </c>
       <c r="T58" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U58" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V58" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W58" s="5" t="inlineStr">
@@ -7915,17 +7915,17 @@
       </c>
       <c r="T59" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U59" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V59" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W59" s="5" t="inlineStr">
@@ -8040,17 +8040,17 @@
       </c>
       <c r="T60" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U60" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V60" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W60" s="5" t="inlineStr">
@@ -8165,17 +8165,17 @@
       </c>
       <c r="T61" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U61" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V61" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W61" s="5" t="inlineStr">
@@ -8290,17 +8290,17 @@
       </c>
       <c r="T62" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U62" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V62" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W62" s="5" t="inlineStr">
@@ -8415,17 +8415,17 @@
       </c>
       <c r="T63" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U63" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V63" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W63" s="5" t="inlineStr">
@@ -8540,17 +8540,17 @@
       </c>
       <c r="T64" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U64" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V64" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W64" s="5" t="inlineStr">
@@ -8665,17 +8665,17 @@
       </c>
       <c r="T65" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U65" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V65" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W65" s="5" t="inlineStr">
@@ -8790,17 +8790,17 @@
       </c>
       <c r="T66" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U66" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V66" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W66" s="5" t="inlineStr">
@@ -8915,17 +8915,17 @@
       </c>
       <c r="T67" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U67" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V67" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W67" s="5" t="inlineStr">
@@ -9040,17 +9040,17 @@
       </c>
       <c r="T68" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U68" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V68" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W68" s="5" t="inlineStr">
@@ -9165,17 +9165,17 @@
       </c>
       <c r="T69" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U69" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V69" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W69" s="5" t="inlineStr">
@@ -9290,17 +9290,17 @@
       </c>
       <c r="T70" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U70" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V70" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W70" s="5" t="inlineStr">
@@ -9415,17 +9415,17 @@
       </c>
       <c r="T71" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U71" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V71" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W71" s="5" t="inlineStr">
@@ -9540,17 +9540,17 @@
       </c>
       <c r="T72" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U72" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V72" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W72" s="5" t="inlineStr">
@@ -9665,17 +9665,17 @@
       </c>
       <c r="T73" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U73" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V73" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W73" s="5" t="inlineStr">
@@ -9790,17 +9790,17 @@
       </c>
       <c r="T74" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U74" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V74" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W74" s="5" t="inlineStr">
@@ -9915,17 +9915,17 @@
       </c>
       <c r="T75" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U75" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V75" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W75" s="5" t="inlineStr">
@@ -10040,17 +10040,17 @@
       </c>
       <c r="T76" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U76" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V76" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W76" s="5" t="inlineStr">
@@ -10165,17 +10165,17 @@
       </c>
       <c r="T77" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U77" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V77" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W77" s="5" t="inlineStr">
@@ -10290,17 +10290,17 @@
       </c>
       <c r="T78" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U78" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V78" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W78" s="5" t="inlineStr">
@@ -10415,17 +10415,17 @@
       </c>
       <c r="T79" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U79" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V79" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W79" s="5" t="inlineStr">
@@ -10540,17 +10540,17 @@
       </c>
       <c r="T80" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U80" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V80" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W80" s="5" t="inlineStr">
@@ -10665,17 +10665,17 @@
       </c>
       <c r="T81" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U81" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V81" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W81" s="5" t="inlineStr">
@@ -10790,17 +10790,17 @@
       </c>
       <c r="T82" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U82" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V82" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W82" s="5" t="inlineStr">
@@ -10915,17 +10915,17 @@
       </c>
       <c r="T83" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U83" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V83" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W83" s="5" t="inlineStr">
@@ -11040,17 +11040,17 @@
       </c>
       <c r="T84" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U84" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V84" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W84" s="5" t="inlineStr">
@@ -11165,17 +11165,17 @@
       </c>
       <c r="T85" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U85" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V85" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W85" s="5" t="inlineStr">
@@ -11290,17 +11290,17 @@
       </c>
       <c r="T86" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U86" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V86" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W86" s="5" t="inlineStr">
@@ -11415,17 +11415,17 @@
       </c>
       <c r="T87" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U87" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V87" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W87" s="5" t="inlineStr">
@@ -11540,17 +11540,17 @@
       </c>
       <c r="T88" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U88" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V88" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W88" s="5" t="inlineStr">
@@ -11665,17 +11665,17 @@
       </c>
       <c r="T89" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U89" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V89" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W89" s="5" t="inlineStr">
@@ -11790,17 +11790,17 @@
       </c>
       <c r="T90" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U90" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V90" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W90" s="5" t="inlineStr">
@@ -11915,17 +11915,17 @@
       </c>
       <c r="T91" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U91" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V91" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W91" s="5" t="inlineStr">
@@ -12040,17 +12040,17 @@
       </c>
       <c r="T92" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U92" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V92" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W92" s="5" t="inlineStr">
@@ -12165,17 +12165,17 @@
       </c>
       <c r="T93" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U93" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V93" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W93" s="5" t="inlineStr">
@@ -12290,17 +12290,17 @@
       </c>
       <c r="T94" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U94" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V94" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W94" s="5" t="inlineStr">
@@ -12415,17 +12415,17 @@
       </c>
       <c r="T95" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U95" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V95" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W95" s="5" t="inlineStr">
@@ -12540,17 +12540,17 @@
       </c>
       <c r="T96" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U96" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V96" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W96" s="5" t="inlineStr">
@@ -12665,17 +12665,17 @@
       </c>
       <c r="T97" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U97" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V97" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W97" s="5" t="inlineStr">
@@ -12790,17 +12790,17 @@
       </c>
       <c r="T98" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U98" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V98" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W98" s="5" t="inlineStr">
@@ -12915,17 +12915,17 @@
       </c>
       <c r="T99" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U99" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V99" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W99" s="5" t="inlineStr">
@@ -13040,17 +13040,17 @@
       </c>
       <c r="T100" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U100" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V100" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W100" s="5" t="inlineStr">
@@ -13165,17 +13165,17 @@
       </c>
       <c r="T101" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U101" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V101" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W101" s="5" t="inlineStr">
@@ -13290,17 +13290,17 @@
       </c>
       <c r="T102" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U102" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V102" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W102" s="5" t="inlineStr">
@@ -13415,17 +13415,17 @@
       </c>
       <c r="T103" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U103" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V103" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W103" s="5" t="inlineStr">
@@ -13540,17 +13540,17 @@
       </c>
       <c r="T104" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U104" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V104" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W104" s="5" t="inlineStr">
@@ -13665,17 +13665,17 @@
       </c>
       <c r="T105" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U105" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V105" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W105" s="5" t="inlineStr">
@@ -13790,17 +13790,17 @@
       </c>
       <c r="T106" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U106" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V106" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W106" s="5" t="inlineStr">
@@ -13915,17 +13915,17 @@
       </c>
       <c r="T107" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U107" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V107" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W107" s="5" t="inlineStr">
@@ -14040,17 +14040,17 @@
       </c>
       <c r="T108" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U108" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V108" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W108" s="5" t="inlineStr">
@@ -14165,17 +14165,17 @@
       </c>
       <c r="T109" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U109" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V109" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W109" s="5" t="inlineStr">
@@ -14290,17 +14290,17 @@
       </c>
       <c r="T110" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U110" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V110" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W110" s="5" t="inlineStr">
@@ -14415,17 +14415,17 @@
       </c>
       <c r="T111" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U111" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V111" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W111" s="5" t="inlineStr">
@@ -14540,17 +14540,17 @@
       </c>
       <c r="T112" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U112" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V112" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W112" s="5" t="inlineStr">
@@ -14665,17 +14665,17 @@
       </c>
       <c r="T113" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U113" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V113" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W113" s="5" t="inlineStr">
@@ -14790,17 +14790,17 @@
       </c>
       <c r="T114" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U114" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V114" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W114" s="5" t="inlineStr">
@@ -14915,17 +14915,17 @@
       </c>
       <c r="T115" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U115" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V115" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W115" s="5" t="inlineStr">
@@ -15040,17 +15040,17 @@
       </c>
       <c r="T116" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U116" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V116" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W116" s="5" t="inlineStr">
@@ -15165,17 +15165,17 @@
       </c>
       <c r="T117" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U117" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V117" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W117" s="5" t="inlineStr">
@@ -15290,17 +15290,17 @@
       </c>
       <c r="T118" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U118" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V118" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W118" s="5" t="inlineStr">
@@ -15415,17 +15415,17 @@
       </c>
       <c r="T119" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U119" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V119" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W119" s="5" t="inlineStr">
@@ -15540,17 +15540,17 @@
       </c>
       <c r="T120" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U120" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V120" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W120" s="5" t="inlineStr">
@@ -15665,17 +15665,17 @@
       </c>
       <c r="T121" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U121" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V121" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W121" s="5" t="inlineStr">
@@ -15790,17 +15790,17 @@
       </c>
       <c r="T122" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U122" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V122" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W122" s="5" t="inlineStr">
@@ -15915,17 +15915,17 @@
       </c>
       <c r="T123" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U123" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V123" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W123" s="5" t="inlineStr">
@@ -16040,17 +16040,17 @@
       </c>
       <c r="T124" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U124" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V124" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W124" s="5" t="inlineStr">
@@ -16165,17 +16165,17 @@
       </c>
       <c r="T125" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U125" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V125" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W125" s="5" t="inlineStr">
@@ -16290,17 +16290,17 @@
       </c>
       <c r="T126" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U126" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V126" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W126" s="5" t="inlineStr">
@@ -16415,17 +16415,17 @@
       </c>
       <c r="T127" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U127" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V127" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W127" s="5" t="inlineStr">
@@ -16540,17 +16540,17 @@
       </c>
       <c r="T128" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U128" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V128" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W128" s="5" t="inlineStr">
@@ -16665,17 +16665,17 @@
       </c>
       <c r="T129" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U129" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V129" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W129" s="5" t="inlineStr">
@@ -16790,17 +16790,17 @@
       </c>
       <c r="T130" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U130" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V130" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W130" s="5" t="inlineStr">
@@ -16915,17 +16915,17 @@
       </c>
       <c r="T131" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U131" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V131" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W131" s="5" t="inlineStr">
@@ -17040,17 +17040,17 @@
       </c>
       <c r="T132" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U132" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V132" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W132" s="5" t="inlineStr">
@@ -17165,17 +17165,17 @@
       </c>
       <c r="T133" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U133" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V133" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W133" s="5" t="inlineStr">
@@ -17290,17 +17290,17 @@
       </c>
       <c r="T134" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U134" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V134" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W134" s="5" t="inlineStr">
@@ -17528,17 +17528,17 @@
       </c>
       <c r="T136" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U136" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V136" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W136" s="5" t="inlineStr">
@@ -17653,17 +17653,17 @@
       </c>
       <c r="T137" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U137" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V137" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W137" s="5" t="inlineStr">
@@ -17778,17 +17778,17 @@
       </c>
       <c r="T138" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U138" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V138" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W138" s="5" t="inlineStr">
@@ -17903,17 +17903,17 @@
       </c>
       <c r="T139" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U139" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V139" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W139" s="5" t="inlineStr">
@@ -18028,17 +18028,17 @@
       </c>
       <c r="T140" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U140" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V140" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W140" s="5" t="inlineStr">
@@ -18153,17 +18153,17 @@
       </c>
       <c r="T141" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U141" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V141" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W141" s="5" t="inlineStr">
@@ -18278,17 +18278,17 @@
       </c>
       <c r="T142" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U142" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V142" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W142" s="5" t="inlineStr">
@@ -18403,17 +18403,17 @@
       </c>
       <c r="T143" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U143" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V143" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W143" s="5" t="inlineStr">
@@ -18528,17 +18528,17 @@
       </c>
       <c r="T144" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="U144" s="5" t="inlineStr">
         <is>
-          <t>00a8fe2</t>
+          <t>19eec7a</t>
         </is>
       </c>
       <c r="V144" s="5" t="inlineStr">
         <is>
-          <t>ip/buffered_axi_lite_uart/tb/scripts/vivado/xsim.log</t>
+          <t>output/balu_ral_session2/tb/scripts/vivado/xsim.log</t>
         </is>
       </c>
       <c r="W144" s="5" t="inlineStr">

</xml_diff>